<commit_message>
Added a note regarding topic of dicussion for group counselling session
</commit_message>
<xml_diff>
--- a/forms/app/group_counseling.xlsx
+++ b/forms/app/group_counseling.xlsx
@@ -1,19 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\D-tree\config-dtree-newrepo\config-dtree\forms\app\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6325"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="survey" sheetId="1" r:id="rId4"/>
-    <sheet state="visible" name="choices" sheetId="2" r:id="rId5"/>
-    <sheet state="visible" name="settings" sheetId="3" r:id="rId6"/>
+    <sheet name="survey" sheetId="1" r:id="rId1"/>
+    <sheet name="choices" sheetId="2" r:id="rId2"/>
+    <sheet name="settings" sheetId="3" r:id="rId3"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="120">
   <si>
     <t>type</t>
   </si>
@@ -381,54 +389,67 @@
   <si>
     <t>data</t>
   </si>
+  <si>
+    <t>note_to_chv</t>
+  </si>
+  <si>
+    <t>&lt;span style="color:#f58a1f;font-weight: bold"&gt;Muhudumu wa afya ya Jamii anaushauriwa kutumia Bango Kitita au Muongozo wa Michezo na mawasiliano kuaandaa mkutano wa kikundi kulingana na uhitaji wa eneo lake, Pia anaweza kuomba muongozo/ushauri kutoka kwa msimamizi wake jinsi ya kuandaa ajenda ya ushauri wa kikundi.&lt;/span&gt;</t>
+  </si>
+  <si>
+    <t>&lt;span style="color:#f58a1f;font-weight: bold"&gt;CHV is advised to use Bangokitita or play and communication guide to prepare for group counseling with regards to the needs of his/her catchment area.He /she can also ask for guidance from his/her supervisor on how to create the agendas for the Group counselling session.&lt;/span&gt;</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="10">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF1D1C1D"/>
       <name val="Slack-Lato"/>
     </font>
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Sans"/>
     </font>
     <font>
-      <sz val="12.0"/>
+      <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="12.0"/>
+      <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Cambria"/>
     </font>
@@ -438,7 +459,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -454,119 +475,84 @@
     </fill>
   </fills>
   <borders count="3">
-    <border/>
     <border>
+      <left/>
       <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="thin">
         <color rgb="FFB2B2B2"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="29">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="2" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -756,23 +742,26 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.75"/>
+  <dimension ref="A1:Z37"/>
+  <sheetFormatPr defaultColWidth="14.40625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="26.43"/>
-    <col customWidth="1" min="3" max="3" width="26.86"/>
-    <col customWidth="1" min="4" max="4" width="31.43"/>
-    <col customWidth="1" min="9" max="9" width="26.14"/>
+    <col min="2" max="2" width="26.40625" customWidth="1"/>
+    <col min="3" max="3" width="26.86328125" customWidth="1"/>
+    <col min="4" max="4" width="31.40625" customWidth="1"/>
+    <col min="9" max="9" width="26.1328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:26" ht="13">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -834,7 +823,7 @@
       <c r="Y1" s="3"/>
       <c r="Z1" s="3"/>
     </row>
-    <row r="2">
+    <row r="2" spans="1:26" ht="13">
       <c r="A2" s="4" t="s">
         <v>17</v>
       </c>
@@ -871,7 +860,7 @@
       <c r="Y2" s="3"/>
       <c r="Z2" s="3"/>
     </row>
-    <row r="3">
+    <row r="3" spans="1:26" ht="13">
       <c r="A3" s="4" t="s">
         <v>17</v>
       </c>
@@ -905,7 +894,7 @@
       <c r="Y3" s="3"/>
       <c r="Z3" s="3"/>
     </row>
-    <row r="4">
+    <row r="4" spans="1:26" ht="13">
       <c r="A4" s="4" t="s">
         <v>21</v>
       </c>
@@ -939,7 +928,7 @@
       <c r="Y4" s="3"/>
       <c r="Z4" s="3"/>
     </row>
-    <row r="5">
+    <row r="5" spans="1:26" ht="13">
       <c r="A5" s="4" t="s">
         <v>21</v>
       </c>
@@ -973,7 +962,7 @@
       <c r="Y5" s="3"/>
       <c r="Z5" s="3"/>
     </row>
-    <row r="6">
+    <row r="6" spans="1:26" ht="13">
       <c r="A6" s="4" t="s">
         <v>21</v>
       </c>
@@ -1007,7 +996,7 @@
       <c r="Y6" s="3"/>
       <c r="Z6" s="3"/>
     </row>
-    <row r="7">
+    <row r="7" spans="1:26" ht="13">
       <c r="A7" s="4" t="s">
         <v>27</v>
       </c>
@@ -1039,7 +1028,7 @@
       <c r="Y7" s="3"/>
       <c r="Z7" s="3"/>
     </row>
-    <row r="8">
+    <row r="8" spans="1:26" ht="13">
       <c r="A8" s="4" t="s">
         <v>27</v>
       </c>
@@ -1071,7 +1060,7 @@
       <c r="Y8" s="3"/>
       <c r="Z8" s="3"/>
     </row>
-    <row r="9">
+    <row r="9" spans="1:26" ht="13">
       <c r="A9" s="4" t="s">
         <v>28</v>
       </c>
@@ -1107,7 +1096,7 @@
       <c r="Y9" s="3"/>
       <c r="Z9" s="3"/>
     </row>
-    <row r="10">
+    <row r="10" spans="1:26" ht="13">
       <c r="A10" s="4" t="s">
         <v>28</v>
       </c>
@@ -1143,7 +1132,7 @@
       <c r="Y10" s="3"/>
       <c r="Z10" s="3"/>
     </row>
-    <row r="11">
+    <row r="11" spans="1:26" ht="13">
       <c r="A11" s="4" t="s">
         <v>28</v>
       </c>
@@ -1179,7 +1168,7 @@
       <c r="Y11" s="3"/>
       <c r="Z11" s="3"/>
     </row>
-    <row r="12">
+    <row r="12" spans="1:26" ht="13">
       <c r="A12" s="8" t="s">
         <v>36</v>
       </c>
@@ -1211,7 +1200,7 @@
       <c r="Y12" s="12"/>
       <c r="Z12" s="12"/>
     </row>
-    <row r="13">
+    <row r="13" spans="1:26" ht="13">
       <c r="A13" s="8" t="s">
         <v>37</v>
       </c>
@@ -1243,7 +1232,7 @@
       <c r="Y13" s="12"/>
       <c r="Z13" s="12"/>
     </row>
-    <row r="14">
+    <row r="14" spans="1:26" ht="13">
       <c r="A14" s="9" t="s">
         <v>38</v>
       </c>
@@ -1272,7 +1261,7 @@
       <c r="R14" s="12"/>
       <c r="S14" s="12"/>
     </row>
-    <row r="15" ht="22.5" customHeight="1">
+    <row r="15" spans="1:26" ht="22.5" customHeight="1">
       <c r="A15" s="9" t="s">
         <v>42</v>
       </c>
@@ -1301,7 +1290,7 @@
       <c r="R15" s="12"/>
       <c r="S15" s="12"/>
     </row>
-    <row r="16">
+    <row r="16" spans="1:26" ht="13">
       <c r="A16" s="9" t="s">
         <v>46</v>
       </c>
@@ -1326,16 +1315,17 @@
       <c r="R16" s="12"/>
       <c r="S16" s="12"/>
     </row>
-    <row r="17">
+    <row r="17" spans="1:17" ht="13">
       <c r="A17" s="14" t="s">
         <v>17</v>
       </c>
       <c r="B17" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="C17" s="14" t="s">
+      <c r="C17" s="27" t="s">
         <v>19</v>
       </c>
+      <c r="D17" s="27"/>
       <c r="E17" s="15"/>
       <c r="F17" s="16"/>
       <c r="G17" s="14" t="s">
@@ -1352,34 +1342,24 @@
       <c r="P17" s="16"/>
       <c r="Q17" s="16"/>
     </row>
-    <row r="18">
-      <c r="A18" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="B18" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="C18" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="D18" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="E18" s="14" t="s">
-        <v>53</v>
+    <row r="18" spans="1:17" s="20" customFormat="1" ht="13">
+      <c r="A18" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="C18" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="D18" s="20" t="s">
+        <v>118</v>
       </c>
       <c r="F18" s="16"/>
-      <c r="G18" s="16"/>
       <c r="H18" s="16"/>
-      <c r="I18" s="17" t="s">
-        <v>54</v>
-      </c>
-      <c r="J18" s="18" t="s">
-        <v>55</v>
-      </c>
-      <c r="K18" s="18" t="s">
-        <v>56</v>
-      </c>
+      <c r="I18" s="16"/>
+      <c r="J18" s="16"/>
+      <c r="K18" s="16"/>
       <c r="L18" s="16"/>
       <c r="M18" s="16"/>
       <c r="N18" s="16"/>
@@ -1387,18 +1367,18 @@
       <c r="P18" s="16"/>
       <c r="Q18" s="16"/>
     </row>
-    <row r="19">
+    <row r="19" spans="1:17" ht="13">
       <c r="A19" s="14" t="s">
         <v>49</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="E19" s="14" t="s">
         <v>53</v>
@@ -1410,10 +1390,10 @@
         <v>54</v>
       </c>
       <c r="J19" s="18" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="K19" s="18" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="L19" s="16"/>
       <c r="M19" s="16"/>
@@ -1422,18 +1402,18 @@
       <c r="P19" s="16"/>
       <c r="Q19" s="16"/>
     </row>
-    <row r="20">
+    <row r="20" spans="1:17" ht="13">
       <c r="A20" s="14" t="s">
         <v>49</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="E20" s="14" t="s">
         <v>53</v>
@@ -1445,10 +1425,10 @@
         <v>54</v>
       </c>
       <c r="J20" s="18" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="K20" s="18" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="L20" s="16"/>
       <c r="M20" s="16"/>
@@ -1457,33 +1437,33 @@
       <c r="P20" s="16"/>
       <c r="Q20" s="16"/>
     </row>
-    <row r="21">
+    <row r="21" spans="1:17" ht="13">
       <c r="A21" s="14" t="s">
-        <v>66</v>
+        <v>49</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="E21" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="F21" s="19"/>
+      <c r="F21" s="16"/>
       <c r="G21" s="16"/>
       <c r="H21" s="16"/>
-      <c r="I21" s="14" t="s">
-        <v>70</v>
+      <c r="I21" s="17" t="s">
+        <v>54</v>
       </c>
       <c r="J21" s="18" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="K21" s="18" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="L21" s="16"/>
       <c r="M21" s="16"/>
@@ -1492,31 +1472,33 @@
       <c r="P21" s="16"/>
       <c r="Q21" s="16"/>
     </row>
-    <row r="22">
+    <row r="22" spans="1:17" ht="13">
       <c r="A22" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="B22" s="20" t="s">
-        <v>73</v>
+        <v>66</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>67</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="E22" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="F22" s="16"/>
+      <c r="F22" s="19"/>
       <c r="G22" s="16"/>
       <c r="H22" s="16"/>
-      <c r="I22" s="16"/>
+      <c r="I22" s="14" t="s">
+        <v>70</v>
+      </c>
       <c r="J22" s="18" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="K22" s="18" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="L22" s="16"/>
       <c r="M22" s="16"/>
@@ -1525,23 +1507,32 @@
       <c r="P22" s="16"/>
       <c r="Q22" s="16"/>
     </row>
-    <row r="23">
+    <row r="23" spans="1:17" ht="13">
       <c r="A23" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="B23" s="14" t="s">
-        <v>78</v>
+        <v>49</v>
+      </c>
+      <c r="B23" s="20" t="s">
+        <v>73</v>
       </c>
       <c r="C23" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="E23" s="14"/>
+        <v>74</v>
+      </c>
+      <c r="D23" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="E23" s="14" t="s">
+        <v>53</v>
+      </c>
       <c r="F23" s="16"/>
       <c r="G23" s="16"/>
       <c r="H23" s="16"/>
       <c r="I23" s="16"/>
-      <c r="J23" s="16"/>
-      <c r="K23" s="16"/>
+      <c r="J23" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="K23" s="18" t="s">
+        <v>77</v>
+      </c>
       <c r="L23" s="16"/>
       <c r="M23" s="16"/>
       <c r="N23" s="16"/>
@@ -1549,32 +1540,24 @@
       <c r="P23" s="16"/>
       <c r="Q23" s="16"/>
     </row>
-    <row r="24">
+    <row r="24" spans="1:17" ht="13">
       <c r="A24" s="14" t="s">
-        <v>79</v>
+        <v>17</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="C24" s="14" t="s">
-        <v>81</v>
-      </c>
-      <c r="D24" s="14" t="s">
-        <v>82</v>
-      </c>
+        <v>78</v>
+      </c>
+      <c r="C24" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="D24" s="27"/>
       <c r="E24" s="14"/>
       <c r="F24" s="16"/>
       <c r="G24" s="16"/>
       <c r="H24" s="16"/>
-      <c r="I24" s="21" t="s">
-        <v>83</v>
-      </c>
-      <c r="J24" s="18" t="s">
-        <v>84</v>
-      </c>
-      <c r="K24" s="18" t="s">
-        <v>85</v>
-      </c>
+      <c r="I24" s="16"/>
+      <c r="J24" s="16"/>
+      <c r="K24" s="16"/>
       <c r="L24" s="16"/>
       <c r="M24" s="16"/>
       <c r="N24" s="16"/>
@@ -1582,18 +1565,18 @@
       <c r="P24" s="16"/>
       <c r="Q24" s="16"/>
     </row>
-    <row r="25">
+    <row r="25" spans="1:17" ht="13">
       <c r="A25" s="14" t="s">
         <v>79</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="E25" s="14"/>
       <c r="F25" s="16"/>
@@ -1615,23 +1598,32 @@
       <c r="P25" s="16"/>
       <c r="Q25" s="16"/>
     </row>
-    <row r="26">
+    <row r="26" spans="1:17" ht="13">
       <c r="A26" s="14" t="s">
-        <v>27</v>
+        <v>79</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>19</v>
+        <v>87</v>
+      </c>
+      <c r="D26" s="14" t="s">
+        <v>88</v>
       </c>
       <c r="E26" s="14"/>
       <c r="F26" s="16"/>
       <c r="G26" s="16"/>
       <c r="H26" s="16"/>
-      <c r="I26" s="14"/>
-      <c r="J26" s="14"/>
-      <c r="K26" s="18"/>
+      <c r="I26" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="J26" s="18" t="s">
+        <v>84</v>
+      </c>
+      <c r="K26" s="18" t="s">
+        <v>85</v>
+      </c>
       <c r="L26" s="16"/>
       <c r="M26" s="16"/>
       <c r="N26" s="16"/>
@@ -1639,16 +1631,17 @@
       <c r="P26" s="16"/>
       <c r="Q26" s="16"/>
     </row>
-    <row r="27">
+    <row r="27" spans="1:17" ht="13">
       <c r="A27" s="14" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>89</v>
-      </c>
-      <c r="C27" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="C27" s="27" t="s">
         <v>19</v>
       </c>
+      <c r="D27" s="27"/>
       <c r="E27" s="14"/>
       <c r="F27" s="16"/>
       <c r="G27" s="16"/>
@@ -1663,32 +1656,24 @@
       <c r="P27" s="16"/>
       <c r="Q27" s="16"/>
     </row>
-    <row r="28">
+    <row r="28" spans="1:17" ht="13">
       <c r="A28" s="14" t="s">
-        <v>79</v>
+        <v>17</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="C28" s="14" t="s">
-        <v>91</v>
-      </c>
-      <c r="D28" s="14" t="s">
-        <v>92</v>
-      </c>
+        <v>89</v>
+      </c>
+      <c r="C28" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="D28" s="27"/>
       <c r="E28" s="14"/>
       <c r="F28" s="16"/>
       <c r="G28" s="16"/>
       <c r="H28" s="16"/>
-      <c r="I28" s="21" t="s">
-        <v>83</v>
-      </c>
-      <c r="J28" s="18" t="s">
-        <v>84</v>
-      </c>
-      <c r="K28" s="18" t="s">
-        <v>85</v>
-      </c>
+      <c r="I28" s="14"/>
+      <c r="J28" s="14"/>
+      <c r="K28" s="18"/>
       <c r="L28" s="16"/>
       <c r="M28" s="16"/>
       <c r="N28" s="16"/>
@@ -1696,18 +1681,18 @@
       <c r="P28" s="16"/>
       <c r="Q28" s="16"/>
     </row>
-    <row r="29">
+    <row r="29" spans="1:17" ht="13">
       <c r="A29" s="14" t="s">
         <v>79</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="D29" s="14" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="E29" s="14"/>
       <c r="F29" s="16"/>
@@ -1729,23 +1714,32 @@
       <c r="P29" s="16"/>
       <c r="Q29" s="16"/>
     </row>
-    <row r="30">
+    <row r="30" spans="1:17" ht="13">
       <c r="A30" s="14" t="s">
-        <v>27</v>
+        <v>79</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>19</v>
+        <v>94</v>
+      </c>
+      <c r="D30" s="14" t="s">
+        <v>95</v>
       </c>
       <c r="E30" s="14"/>
       <c r="F30" s="16"/>
       <c r="G30" s="16"/>
       <c r="H30" s="16"/>
-      <c r="I30" s="16"/>
-      <c r="J30" s="16"/>
-      <c r="K30" s="16"/>
+      <c r="I30" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="J30" s="18" t="s">
+        <v>84</v>
+      </c>
+      <c r="K30" s="18" t="s">
+        <v>85</v>
+      </c>
       <c r="L30" s="16"/>
       <c r="M30" s="16"/>
       <c r="N30" s="16"/>
@@ -1753,16 +1747,17 @@
       <c r="P30" s="16"/>
       <c r="Q30" s="16"/>
     </row>
-    <row r="31">
+    <row r="31" spans="1:17" ht="13">
       <c r="A31" s="14" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="B31" s="14" t="s">
-        <v>96</v>
-      </c>
-      <c r="C31" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="C31" s="27" t="s">
         <v>19</v>
       </c>
+      <c r="D31" s="27"/>
       <c r="E31" s="14"/>
       <c r="F31" s="16"/>
       <c r="G31" s="16"/>
@@ -1777,32 +1772,24 @@
       <c r="P31" s="16"/>
       <c r="Q31" s="16"/>
     </row>
-    <row r="32">
+    <row r="32" spans="1:17" ht="13">
       <c r="A32" s="14" t="s">
-        <v>79</v>
+        <v>17</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>97</v>
-      </c>
-      <c r="C32" s="14" t="s">
-        <v>98</v>
-      </c>
-      <c r="D32" s="14" t="s">
-        <v>99</v>
-      </c>
+        <v>96</v>
+      </c>
+      <c r="C32" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="D32" s="27"/>
       <c r="E32" s="14"/>
       <c r="F32" s="16"/>
       <c r="G32" s="16"/>
       <c r="H32" s="16"/>
-      <c r="I32" s="21" t="s">
-        <v>83</v>
-      </c>
-      <c r="J32" s="18" t="s">
-        <v>84</v>
-      </c>
-      <c r="K32" s="18" t="s">
-        <v>85</v>
-      </c>
+      <c r="I32" s="16"/>
+      <c r="J32" s="16"/>
+      <c r="K32" s="16"/>
       <c r="L32" s="16"/>
       <c r="M32" s="16"/>
       <c r="N32" s="16"/>
@@ -1810,18 +1797,18 @@
       <c r="P32" s="16"/>
       <c r="Q32" s="16"/>
     </row>
-    <row r="33">
+    <row r="33" spans="1:17" ht="13">
       <c r="A33" s="14" t="s">
         <v>79</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="E33" s="14"/>
       <c r="F33" s="16"/>
@@ -1843,18 +1830,18 @@
       <c r="P33" s="16"/>
       <c r="Q33" s="16"/>
     </row>
-    <row r="34">
+    <row r="34" spans="1:17" ht="13">
       <c r="A34" s="14" t="s">
         <v>79</v>
       </c>
       <c r="B34" s="14" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="E34" s="14"/>
       <c r="F34" s="16"/>
@@ -1876,23 +1863,32 @@
       <c r="P34" s="16"/>
       <c r="Q34" s="16"/>
     </row>
-    <row r="35">
+    <row r="35" spans="1:17" ht="13">
       <c r="A35" s="14" t="s">
-        <v>27</v>
+        <v>79</v>
       </c>
       <c r="B35" s="14" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="E35" s="15"/>
+        <v>104</v>
+      </c>
+      <c r="D35" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="E35" s="14"/>
       <c r="F35" s="16"/>
       <c r="G35" s="16"/>
       <c r="H35" s="16"/>
-      <c r="I35" s="16"/>
-      <c r="J35" s="16"/>
-      <c r="K35" s="16"/>
+      <c r="I35" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="J35" s="18" t="s">
+        <v>84</v>
+      </c>
+      <c r="K35" s="18" t="s">
+        <v>85</v>
+      </c>
       <c r="L35" s="16"/>
       <c r="M35" s="16"/>
       <c r="N35" s="16"/>
@@ -1900,18 +1896,18 @@
       <c r="P35" s="16"/>
       <c r="Q35" s="16"/>
     </row>
-    <row r="36">
-      <c r="A36" s="18" t="s">
+    <row r="36" spans="1:17" ht="13">
+      <c r="A36" s="14" t="s">
         <v>27</v>
       </c>
       <c r="B36" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="C36" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="C36" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="D36" s="16"/>
-      <c r="E36" s="16"/>
+      <c r="D36" s="27"/>
+      <c r="E36" s="15"/>
       <c r="F36" s="16"/>
       <c r="G36" s="16"/>
       <c r="H36" s="16"/>
@@ -1925,32 +1921,58 @@
       <c r="P36" s="16"/>
       <c r="Q36" s="16"/>
     </row>
+    <row r="37" spans="1:17" ht="13">
+      <c r="A37" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B37" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="C37" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="D37" s="16"/>
+      <c r="E37" s="16"/>
+      <c r="F37" s="16"/>
+      <c r="G37" s="16"/>
+      <c r="H37" s="16"/>
+      <c r="I37" s="16"/>
+      <c r="J37" s="16"/>
+      <c r="K37" s="16"/>
+      <c r="L37" s="16"/>
+      <c r="M37" s="16"/>
+      <c r="N37" s="16"/>
+      <c r="O37" s="16"/>
+      <c r="P37" s="16"/>
+      <c r="Q37" s="16"/>
+    </row>
   </sheetData>
   <mergeCells count="7">
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="C36:D36"/>
     <mergeCell ref="C17:D17"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C24:D24"/>
     <mergeCell ref="C27:D27"/>
-    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="C28:D28"/>
     <mergeCell ref="C31:D31"/>
-    <mergeCell ref="C35:D35"/>
   </mergeCells>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.75"/>
+  <dimension ref="A1:Z6"/>
+  <sheetFormatPr defaultColWidth="14.40625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="20.57"/>
-    <col customWidth="1" min="3" max="3" width="26.43"/>
+    <col min="2" max="2" width="20.54296875" customWidth="1"/>
+    <col min="3" max="3" width="26.40625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:26">
       <c r="A1" s="22" t="s">
         <v>106</v>
       </c>
@@ -1986,52 +2008,53 @@
       <c r="Y1" s="3"/>
       <c r="Z1" s="3"/>
     </row>
-    <row r="2">
+    <row r="2" spans="1:26" ht="15.75" customHeight="1">
       <c r="A2" s="24"/>
       <c r="B2" s="24"/>
       <c r="C2" s="24"/>
       <c r="D2" s="24"/>
     </row>
-    <row r="3">
+    <row r="3" spans="1:26" ht="15.75" customHeight="1">
       <c r="A3" s="24"/>
       <c r="B3" s="24"/>
       <c r="C3" s="24"/>
       <c r="D3" s="24"/>
     </row>
-    <row r="4">
+    <row r="4" spans="1:26" ht="15.75" customHeight="1">
       <c r="A4" s="24"/>
       <c r="B4" s="24"/>
       <c r="C4" s="24"/>
       <c r="D4" s="24"/>
     </row>
-    <row r="5">
+    <row r="5" spans="1:26" ht="15.75" customHeight="1">
       <c r="A5" s="24"/>
       <c r="B5" s="24"/>
       <c r="C5" s="24"/>
       <c r="D5" s="24"/>
     </row>
-    <row r="6">
+    <row r="6" spans="1:26" ht="15.75" customHeight="1">
       <c r="A6" s="24"/>
       <c r="B6" s="24"/>
       <c r="C6" s="24"/>
       <c r="D6" s="24"/>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.75"/>
+  <dimension ref="A1:Z2"/>
+  <sheetFormatPr defaultColWidth="14.40625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="17.86"/>
+    <col min="1" max="1" width="17.86328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:26" ht="15.75" customHeight="1">
       <c r="A1" s="25" t="s">
         <v>107</v>
       </c>
@@ -2071,13 +2094,14 @@
       <c r="Y1" s="3"/>
       <c r="Z1" s="3"/>
     </row>
-    <row r="2">
+    <row r="2" spans="1:26" ht="15.75" customHeight="1">
       <c r="A2" s="24" t="s">
         <v>113</v>
       </c>
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="28" t="s">
         <v>114</v>
       </c>
+      <c r="C2" s="27"/>
       <c r="D2" s="24" t="s">
         <v>115</v>
       </c>
@@ -2089,6 +2113,6 @@
   <mergeCells count="1">
     <mergeCell ref="B2:C2"/>
   </mergeCells>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>